<commit_message>
month long update before changing and modifying the simEnv project
</commit_message>
<xml_diff>
--- a/dataAcquisition/Motec_MP/channels/channels.xlsx
+++ b/dataAcquisition/Motec_MP/channels/channels.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SimEnv\dataAcquisition\Motec_MP\channels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECAB1560-0CCD-40E4-A9D2-08C89FD4685C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FCFA652-5F52-485E-9CC6-5597A59912F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="23385" activeTab="1" xr2:uid="{6EEC8272-D558-43BF-A2F2-0B52778D7332}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="23385" xr2:uid="{6EEC8272-D558-43BF-A2F2-0B52778D7332}"/>
   </bookViews>
   <sheets>
     <sheet name="channels" sheetId="2" r:id="rId1"/>
     <sheet name="gatedChannels" sheetId="3" r:id="rId2"/>
     <sheet name="matlabCreatedGates" sheetId="5" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">channels!$B$1:$B$1034</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">channels!$B$1:$B$1056</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1156" uniqueCount="1097">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1178" uniqueCount="1160">
   <si>
     <t xml:space="preserve">Beacon                </t>
   </si>
@@ -2965,12 +2966,6 @@
     <t xml:space="preserve">Reference Lap Time Reset          </t>
   </si>
   <si>
-    <t xml:space="preserve">TPM1S XX DIAG VEH MOVING          </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cond Full Throttle Reset          </t>
-  </si>
-  <si>
     <t xml:space="preserve">Cond Over Rev                     </t>
   </si>
   <si>
@@ -3046,21 +3041,9 @@
     <t>rTyreRL_VCH_P_FZ_C</t>
   </si>
   <si>
-    <t>exitGateVCH.*RL_SlipVCH</t>
-  </si>
-  <si>
     <t>RL_SlipVCH_exitGate</t>
   </si>
   <si>
-    <t>Gate_LowSpeed.*Ground_Speed</t>
-  </si>
-  <si>
-    <t>Gate_MidSpeed.*Ground_Speed</t>
-  </si>
-  <si>
-    <t>Gate_HighSpeed.*Ground_Speed</t>
-  </si>
-  <si>
     <t>Ground_Speed_low_VCH</t>
   </si>
   <si>
@@ -3079,147 +3062,18 @@
     <t>Lat_High_VCH</t>
   </si>
   <si>
-    <t>brakingGateVCH.*Acceleration_X_Filt</t>
-  </si>
-  <si>
-    <t>entryGateVCH.*Acceleration_X_Filt</t>
-  </si>
-  <si>
     <t>Braking_gLong</t>
   </si>
   <si>
     <t>Entry_gLong</t>
   </si>
   <si>
-    <t>Gate_LowSpeed.*abs(Acceleration_Y_Filt)</t>
-  </si>
-  <si>
-    <t>Gate_MidSpeed.*abs(Acceleration_Y_Filt)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gate_HighSpeed.*abs(Acceleration_Y_Filt)        </t>
-  </si>
-  <si>
-    <t>Parity_Speed .* Ground_Speed</t>
-  </si>
-  <si>
     <t>Parity_Speed</t>
   </si>
   <si>
     <t>fullThrottleGroundSpeed</t>
   </si>
   <si>
-    <t>straightGateVCH.*Ground_Speed</t>
-  </si>
-  <si>
-    <t>brakingGateVCH .* CLa_SCz_VCH_KIN</t>
-  </si>
-  <si>
-    <t>entryGateVCH .* CLa_SCz_VCH_KIN</t>
-  </si>
-  <si>
-    <t>midCrnGateVCH .* CLa_SCz_VCH_KIN</t>
-  </si>
-  <si>
-    <t>exitGateVCH .* CLa_SCz_VCH_KIN</t>
-  </si>
-  <si>
-    <t>Gate_LowSpeed.*CDa_SCx_VCH_KIN</t>
-  </si>
-  <si>
-    <t>Gate_MidSpeed.*CDa_SCx_VCH_KIN</t>
-  </si>
-  <si>
-    <t>Gate_HighSpeed.*CDa_SCx_VCH_KIN</t>
-  </si>
-  <si>
-    <t>ParityMaskVCH.*CDa_SCx_VCH_KIN</t>
-  </si>
-  <si>
-    <t>AB_FRT_VCH_KIN.*brakingGateVCH</t>
-  </si>
-  <si>
-    <t>AB_FRT_VCH_KIN.*entryGateVCH</t>
-  </si>
-  <si>
-    <t>AB_FRT_VCH_KIN.*midCrnGateVCH</t>
-  </si>
-  <si>
-    <t>AB_FRT_VCH_KIN.*exitGateVCH</t>
-  </si>
-  <si>
-    <t>EFF_VCH_KIN.*brakingGateVCH</t>
-  </si>
-  <si>
-    <t>EFF_VCH_KIN.*entryGateVCH</t>
-  </si>
-  <si>
-    <t>EFF_VCH_KIN.*midCrnGateVCH</t>
-  </si>
-  <si>
-    <t>EFF_VCH_KIN.*exitGateVCH</t>
-  </si>
-  <si>
-    <t>CSa_Scy_VCH_KIN.*entryGateVCH</t>
-  </si>
-  <si>
-    <t>CSa_Scy_VCH_KIN.*midCrnGateVCH</t>
-  </si>
-  <si>
-    <t>brakingGateVCH .*CLz_MEAS</t>
-  </si>
-  <si>
-    <t>entryGateVCH .* CLz_MEAS</t>
-  </si>
-  <si>
-    <t>midCrnGateVCH .* CLz_MEAS</t>
-  </si>
-  <si>
-    <t>exitGateVCH .* CLz_MEAS</t>
-  </si>
-  <si>
-    <t>Gate_LowSpeed.* CDx_MEAS</t>
-  </si>
-  <si>
-    <t>Gate_HighSpeed.* CDx_MEAS</t>
-  </si>
-  <si>
-    <t>Gate_MidSpeed.* CDx_MEAS</t>
-  </si>
-  <si>
-    <t>ParityMaskVCH.* CDx_MEAS</t>
-  </si>
-  <si>
-    <t>ABf_MEAS.*brakingGateVCH</t>
-  </si>
-  <si>
-    <t>ABf_MEAS.*entryGateVCH</t>
-  </si>
-  <si>
-    <t>ABf_MEAS.*midCrnGateVCH</t>
-  </si>
-  <si>
-    <t>ABf_MEAS.*exitGateVCH</t>
-  </si>
-  <si>
-    <t>EFF_MEAS.*brakingGateVCH</t>
-  </si>
-  <si>
-    <t>EFF_MEAS.*entryGateVCH</t>
-  </si>
-  <si>
-    <t>EFF_MEAS.*midCrnGateVCH</t>
-  </si>
-  <si>
-    <t>EFF_MEAS.*exitGateVCH</t>
-  </si>
-  <si>
-    <t>CLy_MEAS.*entryGateVCH</t>
-  </si>
-  <si>
-    <t>CLy_MEAS.*midCrnGateVCH</t>
-  </si>
-  <si>
     <t>CLz_Braking_Gate_Meas</t>
   </si>
   <si>
@@ -3328,10 +3182,346 @@
     <t>Cy_Mid_Kin</t>
   </si>
   <si>
-    <t>Clz_Braking_Gate_Meas</t>
-  </si>
-  <si>
-    <t>Clz_Braking_Gate_Kin</t>
+    <t>Comms CAN 15 Diag</t>
+  </si>
+  <si>
+    <t>Driver ID Volts</t>
+  </si>
+  <si>
+    <t>Over Rev Engine Threshold</t>
+  </si>
+  <si>
+    <t>Over Rev Throttle Threshold</t>
+  </si>
+  <si>
+    <t>TPM1S XX WS CONFIRMED</t>
+  </si>
+  <si>
+    <t>Timer Stall Msg Tx</t>
+  </si>
+  <si>
+    <t>X2 Car Number</t>
+  </si>
+  <si>
+    <t>X2 Gap Ahead</t>
+  </si>
+  <si>
+    <t>X2 RC Count Down</t>
+  </si>
+  <si>
+    <t>X2 RLP BaseLink Connected</t>
+  </si>
+  <si>
+    <t>X2 RLP Flag</t>
+  </si>
+  <si>
+    <t>X2 RLP GPS Epoch Time</t>
+  </si>
+  <si>
+    <t>X2 RLP Heartbeat</t>
+  </si>
+  <si>
+    <t>X2 RLP RF RSSI dBm</t>
+  </si>
+  <si>
+    <t>X2 Stalled Left</t>
+  </si>
+  <si>
+    <t>X2 Stalled Right</t>
+  </si>
+  <si>
+    <t>X2 Stalled Warning</t>
+  </si>
+  <si>
+    <t>X2 Timing Session Time Rem</t>
+  </si>
+  <si>
+    <t>Comms CAN 16 Diag</t>
+  </si>
+  <si>
+    <t>Comms CAN 17 Diag</t>
+  </si>
+  <si>
+    <t>Comms CAN 18 Diag</t>
+  </si>
+  <si>
+    <t>Comms CAN 19 Diag</t>
+  </si>
+  <si>
+    <t>Cond Stalled</t>
+  </si>
+  <si>
+    <t>Driver ID Latched</t>
+  </si>
+  <si>
+    <t>Gate_Exit_VCH.*Slip_RL_VCH</t>
+  </si>
+  <si>
+    <t>Gate_Low_Speed_VCH.*Ground_Speed</t>
+  </si>
+  <si>
+    <t>Gate_Mid_Speed_VCH.*Ground_Speed</t>
+  </si>
+  <si>
+    <t>Gate_High_Speed_VCH.*Ground_Speed</t>
+  </si>
+  <si>
+    <t>Gate_Low_Speed_VCH.*abs(Acceleration_Y_Filt)</t>
+  </si>
+  <si>
+    <t>Gate_Mid_Speed_VCH.*abs(Acceleration_Y_Filt)</t>
+  </si>
+  <si>
+    <t>Gate_High_Speed_VCH.*abs(Acceleration_Y_Filt)</t>
+  </si>
+  <si>
+    <t>Gate_Braking_VCH.*Acceleration_X_Filt</t>
+  </si>
+  <si>
+    <t>Gate_Entry_VCH.*Acceleration_X_Filt</t>
+  </si>
+  <si>
+    <t>Gate_Braking_VCH.*Aero_Cz_VCH_KIN</t>
+  </si>
+  <si>
+    <t>Gate_Entry_VCH.*Aero_Cz_VCH_KIN</t>
+  </si>
+  <si>
+    <t>Gate_Mid_Corner_VCH.*Aero_Cz_VCH_KIN</t>
+  </si>
+  <si>
+    <t>Gate_Exit_VCH.*Aero_Cz_VCH_KIN</t>
+  </si>
+  <si>
+    <t>Parity_Speed.*Ground_Speed</t>
+  </si>
+  <si>
+    <t>Gate_Low_Speed_VCH.*Aero_Cx_VCH_KIN</t>
+  </si>
+  <si>
+    <t>Gate_Mid_Speed_VCH.*Aero_Cx_VCH_KIN</t>
+  </si>
+  <si>
+    <t>Gate_High_Speed_VCH.*Aero_Cx_VCH_KIN</t>
+  </si>
+  <si>
+    <t>Gate_Parity_VCH.*Aero_Cx_VCH_KIN</t>
+  </si>
+  <si>
+    <t>Aero_Balance_Front_VCH_KIN.*Gate_Braking_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Balance_Front_VCH_KIN.*Gate_Entry_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Balance_Front_VCH_KIN.*Gate_Mid_Corner_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Balance_Front_VCH_KIN.*Gate_Exit_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Efficiency_VCH_KIN.*Gate_Braking_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Efficiency_VCH_KIN.*Gate_Entry_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Efficiency_VCH_KIN.*Gate_Mid_Corner_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Efficiency_VCH_KIN.*Gate_Exit_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Cy_VCH_KIN.*Gate_Entry_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Cy_VCH_KIN.*Gate_Mid_Corner_VCH</t>
+  </si>
+  <si>
+    <t>Gate_Straight_VCH.*Ground_Speed</t>
+  </si>
+  <si>
+    <t>Gate_Braking_VCH.*Aero_Cz_VCH_MEAS</t>
+  </si>
+  <si>
+    <t>Gate_Entry_VCH.*Aero_Cz_VCH_MEAS</t>
+  </si>
+  <si>
+    <t>Gate_Mid_Corner_VCH.*Aero_Cz_VCH_MEAS</t>
+  </si>
+  <si>
+    <t>Gate_Exit_VCH.*Aero_Cz_VCH_MEAS</t>
+  </si>
+  <si>
+    <t>Gate_Low_Speed_VCH.*Aero_Cx_VCH_MEAS</t>
+  </si>
+  <si>
+    <t>Gate_Mid_Speed_VCH.*Aero_Cx_VCH_MEAS</t>
+  </si>
+  <si>
+    <t>Gate_High_Speed_VCH.*Aero_Cx_VCH_MEAS</t>
+  </si>
+  <si>
+    <t>Gate_Parity_VCH.*Aero_Cx_VCH_MEAS</t>
+  </si>
+  <si>
+    <t>Aero_Balance_Front_VCH_MEAS.*Gate_Braking_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Balance_Front_VCH_MEAS.*Gate_Entry_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Balance_Front_VCH_MEAS.*Gate_Mid_Corner_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Balance_Front_VCH_MEAS.*Gate_Exit_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Efficiency_VCH_MEAS.*Gate_Braking_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Efficiency_VCH_MEAS.*Gate_Entry_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Efficiency_VCH_MEAS.*Gate_Mid_Corner_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Efficiency_VCH_MEAS.*Gate_Exit_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Cz_VCH_MEAS.*Gate_Entry_VCH</t>
+  </si>
+  <si>
+    <t>Aero_Cz_VCH_MEAS.*Gate_Mid_Corner_VCH</t>
+  </si>
+  <si>
+    <t>RA_Slip_ExitGate</t>
+  </si>
+  <si>
+    <t>Low_Speed_VCH</t>
+  </si>
+  <si>
+    <t>Med_Speed_VCH</t>
+  </si>
+  <si>
+    <t>Hgh_Speed_VCH</t>
+  </si>
+  <si>
+    <t>Low_Lat_VCH</t>
+  </si>
+  <si>
+    <t>Med_Lat_VCH</t>
+  </si>
+  <si>
+    <t>High_lat_VCH</t>
+  </si>
+  <si>
+    <t>X_Accel_BRK_Gate</t>
+  </si>
+  <si>
+    <t>X_Accel_ENT_Gate</t>
+  </si>
+  <si>
+    <t>Cz_MEAS_BRK_Gate</t>
+  </si>
+  <si>
+    <t>Cz_MEAS_ENT_Gate</t>
+  </si>
+  <si>
+    <t>Cz_MEAS_MED_Gate</t>
+  </si>
+  <si>
+    <t>LOW_SPD_Cx_KIN</t>
+  </si>
+  <si>
+    <t>MED_SPD_Cx_KIN</t>
+  </si>
+  <si>
+    <t>HGH_SPD_Cx_KIN</t>
+  </si>
+  <si>
+    <t>PAR_SPD_Cx_KIN</t>
+  </si>
+  <si>
+    <t>ABF_BRK_KIN</t>
+  </si>
+  <si>
+    <t>ABF_ENT_KIN</t>
+  </si>
+  <si>
+    <t>ABF_CRN_KIN</t>
+  </si>
+  <si>
+    <t>ABF_EXT_KIN</t>
+  </si>
+  <si>
+    <t>EFF_EXT_KIN</t>
+  </si>
+  <si>
+    <t>EFF_ENT_KIN</t>
+  </si>
+  <si>
+    <t>EFF_CRN_KIN</t>
+  </si>
+  <si>
+    <t>Cy_ENT_KIN</t>
+  </si>
+  <si>
+    <t>Cy_CRN_KIN</t>
+  </si>
+  <si>
+    <t>STR_SPD</t>
+  </si>
+  <si>
+    <t>Cz_BRK_MEAS</t>
+  </si>
+  <si>
+    <t>Cz_ENT_MEAS</t>
+  </si>
+  <si>
+    <t>Cz_CRN_MEAS</t>
+  </si>
+  <si>
+    <t>Cz_EXT_MEAS</t>
+  </si>
+  <si>
+    <t>LOW_SPD_Cx_MEAS</t>
+  </si>
+  <si>
+    <t>MED_SPD_Cx_MEAS</t>
+  </si>
+  <si>
+    <t>HGH_SPD_Cx_MEAS</t>
+  </si>
+  <si>
+    <t>PAR_SPD_Cx_MEAS</t>
+  </si>
+  <si>
+    <t>ABF_BRK_MEAS</t>
+  </si>
+  <si>
+    <t>ABF_ENT_MEAS</t>
+  </si>
+  <si>
+    <t>ABF_CRN_MEAS</t>
+  </si>
+  <si>
+    <t>ABF_EXT_MEAS</t>
+  </si>
+  <si>
+    <t>EFF_EXT_MEAS</t>
+  </si>
+  <si>
+    <t>EFF_ENT_MEAS</t>
+  </si>
+  <si>
+    <t>EFF_CRN_MEAS</t>
+  </si>
+  <si>
+    <t>Cy_ENT_MEAS</t>
+  </si>
+  <si>
+    <t>Cy_CRN_MEAS</t>
   </si>
 </sst>
 </file>
@@ -3347,7 +3537,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3357,6 +3547,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79995117038483843"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3373,9 +3569,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3710,7 +3907,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCA4F88A-3EEB-45AF-91DF-E65A060D6362}">
-  <dimension ref="A1:E1043"/>
+  <dimension ref="A1:E1048"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.42578125" bestFit="1" customWidth="1"/>
@@ -3719,19 +3916,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
       <c r="B1" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
       <c r="C1" t="s">
+        <v>989</v>
+      </c>
+      <c r="D1" t="s">
+        <v>990</v>
+      </c>
+      <c r="E1" t="s">
         <v>991</v>
-      </c>
-      <c r="D1" t="s">
-        <v>992</v>
-      </c>
-      <c r="E1" t="s">
-        <v>993</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -11632,7 +11829,7 @@
     </row>
     <row r="977" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A977" t="s">
-        <v>975</v>
+        <v>1046</v>
       </c>
       <c r="B977">
         <v>0</v>
@@ -11640,7 +11837,7 @@
     </row>
     <row r="978" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A978" t="s">
-        <v>976</v>
+        <v>1064</v>
       </c>
       <c r="B978">
         <v>0</v>
@@ -11648,526 +11845,188 @@
     </row>
     <row r="979" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A979" t="s">
-        <v>982</v>
+        <v>1065</v>
       </c>
       <c r="B979">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="980" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A980" t="s">
-        <v>979</v>
+        <v>1066</v>
       </c>
       <c r="B980">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="981" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A981" t="s">
-        <v>980</v>
+        <v>1067</v>
       </c>
       <c r="B981">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="982" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A982" t="s">
-        <v>981</v>
+        <v>1068</v>
       </c>
       <c r="B982">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="983" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A983" t="s">
-        <v>983</v>
+        <v>1069</v>
       </c>
       <c r="B983">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="984" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A984" t="s">
-        <v>984</v>
+        <v>1047</v>
       </c>
       <c r="B984">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="985" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A985" t="s">
-        <v>985</v>
+        <v>1048</v>
       </c>
       <c r="B985">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="986" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A986" t="s">
-        <v>986</v>
+        <v>1049</v>
       </c>
       <c r="B986">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="987" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A987" t="s">
-        <v>987</v>
+        <v>1050</v>
       </c>
       <c r="B987">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="988" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A988" t="s">
-        <v>988</v>
+        <v>1051</v>
       </c>
       <c r="B988">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="989" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A989" t="s">
-        <v>989</v>
+        <v>1052</v>
       </c>
       <c r="B989">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="990" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A990" t="s">
-        <v>990</v>
+        <v>1053</v>
       </c>
       <c r="B990">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="991" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A991" t="s">
-        <v>995</v>
+        <v>1054</v>
       </c>
       <c r="B991">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="992" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A992" t="s">
-        <v>996</v>
+        <v>1055</v>
       </c>
       <c r="B992">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="993" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A993" t="s">
-        <v>997</v>
+        <v>1056</v>
       </c>
       <c r="B993">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="994" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A994" t="s">
-        <v>998</v>
+        <v>1057</v>
       </c>
       <c r="B994">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="995" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A995" t="s">
-        <v>999</v>
+        <v>1058</v>
       </c>
       <c r="B995">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="996" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A996" t="s">
-        <v>1000</v>
+        <v>1059</v>
       </c>
       <c r="B996">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="997" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A997" t="s">
-        <v>1002</v>
+        <v>1060</v>
       </c>
       <c r="B997">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="998" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A998" t="s">
-        <v>1006</v>
+        <v>1061</v>
       </c>
       <c r="B998">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="999" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A999" t="s">
-        <v>1007</v>
+        <v>1062</v>
       </c>
       <c r="B999">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1000" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1000" t="s">
-        <v>1008</v>
+        <v>1063</v>
       </c>
       <c r="B1000">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1001" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1001" t="s">
-        <v>1009</v>
-      </c>
-      <c r="B1001">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1002" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1002" t="s">
-        <v>1010</v>
-      </c>
-      <c r="B1002">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1003" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1003" t="s">
-        <v>1011</v>
-      </c>
-      <c r="B1003">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1004" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1004" t="s">
-        <v>1014</v>
-      </c>
-      <c r="B1004">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1005" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1005" t="s">
-        <v>1015</v>
-      </c>
-      <c r="B1005">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1006" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1006" s="1" t="s">
-        <v>1077</v>
-      </c>
-      <c r="B1006">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1007" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1007" t="s">
-        <v>1078</v>
-      </c>
-      <c r="B1007">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1008" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1008" t="s">
-        <v>1079</v>
-      </c>
-      <c r="B1008">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1009" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1009" t="s">
-        <v>1080</v>
-      </c>
-      <c r="B1009">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1010" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1010" t="s">
-        <v>1020</v>
-      </c>
-      <c r="B1010">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1011" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1011" t="s">
-        <v>1081</v>
-      </c>
-      <c r="B1011">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1012" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1012" t="s">
-        <v>1082</v>
-      </c>
-      <c r="B1012">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1013" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1013" t="s">
-        <v>1083</v>
-      </c>
-      <c r="B1013">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1014" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1014" t="s">
-        <v>1084</v>
-      </c>
-      <c r="B1014">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1015" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1015" t="s">
-        <v>1085</v>
-      </c>
-      <c r="B1015">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1016" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1016" t="s">
-        <v>1086</v>
-      </c>
-      <c r="B1016">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1017" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1017" t="s">
-        <v>1087</v>
-      </c>
-      <c r="B1017">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1018" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1018" t="s">
-        <v>1088</v>
-      </c>
-      <c r="B1018">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1019" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1019" t="s">
-        <v>1089</v>
-      </c>
-      <c r="B1019">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1020" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1020" t="s">
-        <v>1090</v>
-      </c>
-      <c r="B1020">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1021" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1021" t="s">
-        <v>1091</v>
-      </c>
-      <c r="B1021">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1022" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1022" t="s">
-        <v>1092</v>
-      </c>
-      <c r="B1022">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1023" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1023" t="s">
-        <v>1093</v>
-      </c>
-      <c r="B1023">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1024" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1024" t="s">
-        <v>1094</v>
-      </c>
-      <c r="B1024">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1025" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1025" t="s">
-        <v>1021</v>
-      </c>
-      <c r="B1025">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1026" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1026" s="1" t="s">
-        <v>1059</v>
-      </c>
-      <c r="B1026">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1027" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1027" t="s">
-        <v>1060</v>
-      </c>
-      <c r="B1027">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1028" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1028" t="s">
-        <v>1061</v>
-      </c>
-      <c r="B1028">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1029" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1029" t="s">
-        <v>1062</v>
-      </c>
-      <c r="B1029">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1030" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1030" t="s">
-        <v>1063</v>
-      </c>
-      <c r="B1030">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1031" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1031" t="s">
-        <v>1064</v>
-      </c>
-      <c r="B1031">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1032" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1032" t="s">
-        <v>1065</v>
-      </c>
-      <c r="B1032">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1033" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1033" t="s">
-        <v>1066</v>
-      </c>
-      <c r="B1033">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1034" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1034" t="s">
-        <v>1067</v>
-      </c>
-      <c r="B1034">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1035" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1035" t="s">
-        <v>1068</v>
-      </c>
-      <c r="B1035">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1036" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1036" t="s">
-        <v>1069</v>
-      </c>
-      <c r="B1036">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1037" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1037" t="s">
-        <v>1070</v>
-      </c>
-      <c r="B1037">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1038" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1038" t="s">
-        <v>1071</v>
-      </c>
-      <c r="B1038">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1039" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1039" t="s">
-        <v>1072</v>
-      </c>
-      <c r="B1039">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1040" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1040" t="s">
-        <v>1074</v>
-      </c>
-      <c r="B1040">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1041" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1041" t="s">
-        <v>1073</v>
-      </c>
-      <c r="B1041">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1042" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1042" t="s">
-        <v>1075</v>
-      </c>
-      <c r="B1042">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1043" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1043" t="s">
-        <v>1076</v>
-      </c>
-      <c r="B1043">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1028" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1028" s="1"/>
+    </row>
+    <row r="1048" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1048" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:B1034" xr:uid="{DCA4F88A-3EEB-45AF-91DF-E65A060D6362}"/>
+  <autoFilter ref="B1:B1056" xr:uid="{DCA4F88A-3EEB-45AF-91DF-E65A060D6362}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
@@ -12193,389 +12052,389 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
       <c r="B1" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1001</v>
+        <v>1070</v>
       </c>
       <c r="B2" t="s">
-        <v>1002</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1003</v>
+        <v>1071</v>
       </c>
       <c r="B3" t="s">
-        <v>1006</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1004</v>
+        <v>1072</v>
       </c>
       <c r="B4" t="s">
-        <v>1007</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>1005</v>
+        <v>1073</v>
       </c>
       <c r="B5" t="s">
-        <v>1008</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>1016</v>
+        <v>1074</v>
       </c>
       <c r="B6" t="s">
-        <v>1009</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>1017</v>
+        <v>1075</v>
       </c>
       <c r="B7" t="s">
-        <v>1010</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>1018</v>
+        <v>1076</v>
       </c>
       <c r="B8" t="s">
-        <v>1011</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>1012</v>
+        <v>1077</v>
       </c>
       <c r="B9" t="s">
-        <v>1014</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>1013</v>
+        <v>1078</v>
       </c>
       <c r="B10" t="s">
-        <v>1015</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>1023</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>1096</v>
+        <v>1079</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>1126</v>
       </c>
       <c r="C11" s="1"/>
       <c r="E11" s="1"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>1024</v>
+        <v>1080</v>
       </c>
       <c r="B12" t="s">
-        <v>1078</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>1025</v>
+        <v>1081</v>
       </c>
       <c r="B13" t="s">
-        <v>1079</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>1026</v>
+        <v>1082</v>
       </c>
       <c r="B14" t="s">
-        <v>1080</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>1019</v>
+        <v>1083</v>
       </c>
       <c r="B15" t="s">
-        <v>1020</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>1027</v>
+        <v>1084</v>
       </c>
       <c r="B16" t="s">
-        <v>1081</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>1028</v>
+        <v>1085</v>
       </c>
       <c r="B17" t="s">
-        <v>1082</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>1029</v>
+        <v>1086</v>
       </c>
       <c r="B18" t="s">
-        <v>1083</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>1030</v>
+        <v>1087</v>
       </c>
       <c r="B19" t="s">
-        <v>1084</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>1031</v>
+        <v>1088</v>
       </c>
       <c r="B20" t="s">
-        <v>1085</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>1032</v>
+        <v>1089</v>
       </c>
       <c r="B21" t="s">
-        <v>1086</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>1033</v>
+        <v>1090</v>
       </c>
       <c r="B22" t="s">
-        <v>1087</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>1034</v>
+        <v>1091</v>
       </c>
       <c r="B23" t="s">
-        <v>1088</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>1035</v>
+        <v>1092</v>
       </c>
       <c r="B24" t="s">
-        <v>1089</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>1036</v>
+        <v>1093</v>
       </c>
       <c r="B25" t="s">
-        <v>1090</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>1037</v>
+        <v>1094</v>
       </c>
       <c r="B26" t="s">
-        <v>1091</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>1038</v>
+        <v>1095</v>
       </c>
       <c r="B27" t="s">
-        <v>1092</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>1039</v>
+        <v>1096</v>
       </c>
       <c r="B28" t="s">
-        <v>1093</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>1040</v>
+        <v>1097</v>
       </c>
       <c r="B29" t="s">
-        <v>1094</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>1022</v>
+        <v>1098</v>
       </c>
       <c r="B30" t="s">
-        <v>1021</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>1041</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>1095</v>
+        <v>1099</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>1143</v>
       </c>
       <c r="D31" s="1"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>1042</v>
+        <v>1100</v>
       </c>
       <c r="B32" t="s">
-        <v>1060</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>1043</v>
+        <v>1101</v>
       </c>
       <c r="B33" t="s">
-        <v>1061</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>1044</v>
+        <v>1102</v>
       </c>
       <c r="B34" t="s">
-        <v>1062</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>1045</v>
+        <v>1103</v>
       </c>
       <c r="B35" t="s">
-        <v>1063</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>1047</v>
+        <v>1104</v>
       </c>
       <c r="B36" t="s">
-        <v>1064</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>1046</v>
+        <v>1105</v>
       </c>
       <c r="B37" t="s">
-        <v>1065</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>1048</v>
+        <v>1106</v>
       </c>
       <c r="B38" t="s">
-        <v>1066</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>1049</v>
+        <v>1107</v>
       </c>
       <c r="B39" t="s">
-        <v>1067</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>1050</v>
+        <v>1108</v>
       </c>
       <c r="B40" t="s">
-        <v>1068</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>1051</v>
+        <v>1109</v>
       </c>
       <c r="B41" t="s">
-        <v>1069</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>1052</v>
+        <v>1110</v>
       </c>
       <c r="B42" t="s">
-        <v>1070</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>1053</v>
+        <v>1111</v>
       </c>
       <c r="B43" t="s">
-        <v>1071</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>1054</v>
+        <v>1112</v>
       </c>
       <c r="B44" t="s">
-        <v>1072</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>1055</v>
+        <v>1113</v>
       </c>
       <c r="B45" t="s">
-        <v>1074</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>1056</v>
+        <v>1114</v>
       </c>
       <c r="B46" t="s">
-        <v>1073</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>1057</v>
+        <v>1115</v>
       </c>
       <c r="B47" t="s">
-        <v>1075</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>1058</v>
+        <v>1116</v>
       </c>
       <c r="B48" t="s">
-        <v>1076</v>
+        <v>1159</v>
       </c>
     </row>
   </sheetData>
@@ -12594,67 +12453,597 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>981</v>
+        <v>979</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>986</v>
+        <v>984</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>987</v>
+        <v>985</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>1008</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9F049BF-4851-41B8-B67B-226B98976C58}">
+  <dimension ref="A1:B65"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>980</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>977</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>978</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>979</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>981</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>982</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>983</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>984</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>985</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>986</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>987</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>988</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>993</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>994</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>995</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>996</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>997</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>998</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>999</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>1002</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>1007</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>1031</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>1034</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>1036</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>1039</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>1040</v>
+      </c>
+      <c r="B41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>1041</v>
+      </c>
+      <c r="B42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>1042</v>
+      </c>
+      <c r="B43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>1044</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="1" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>1011</v>
+      </c>
+      <c r="B49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>1018</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>1019</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
         <v>1020</v>
+      </c>
+      <c r="B58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>1023</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>1024</v>
+      </c>
+      <c r="B63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>1026</v>
+      </c>
+      <c r="B64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B65">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>